<commit_message>
Reorder staff display order in staff_master.csv and request sheet
Staff order changed to: 上口, 板倉, 山田, 高山, 宮路, 若尾, 永田, 鷹野, 大野,
織田, 金上, 藤田 (groups the three 機能訓練指導員 staff together). Regenerated
templates/2026年_シフト希望入力.xlsx to match the new column order.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VNXq9we8b5GmQGFQzTj2KK
</commit_message>
<xml_diff>
--- a/templates/2026年_シフト希望入力.xlsx
+++ b/templates/2026年_シフト希望入力.xlsx
@@ -779,57 +779,57 @@
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
+          <t>板倉芽生</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
           <t>山田恵美</t>
         </is>
       </c>
-      <c r="E3" s="10" t="inlineStr">
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>高山岳</t>
+        </is>
+      </c>
+      <c r="G3" s="10" t="inlineStr">
+        <is>
+          <t>宮路愛</t>
+        </is>
+      </c>
+      <c r="H3" s="10" t="inlineStr">
+        <is>
+          <t>若尾まい</t>
+        </is>
+      </c>
+      <c r="I3" s="10" t="inlineStr">
         <is>
           <t>永田千尋</t>
         </is>
       </c>
-      <c r="F3" s="10" t="inlineStr">
+      <c r="J3" s="10" t="inlineStr">
         <is>
           <t>鷹野かおり</t>
         </is>
       </c>
-      <c r="G3" s="10" t="inlineStr">
-        <is>
-          <t>若尾まい</t>
-        </is>
-      </c>
-      <c r="H3" s="10" t="inlineStr">
+      <c r="K3" s="10" t="inlineStr">
         <is>
           <t>大野リカ子</t>
         </is>
       </c>
-      <c r="I3" s="10" t="inlineStr">
+      <c r="L3" s="10" t="inlineStr">
         <is>
           <t>織田陽子</t>
         </is>
       </c>
-      <c r="J3" s="10" t="inlineStr">
-        <is>
-          <t>板倉芽生</t>
-        </is>
-      </c>
-      <c r="K3" s="10" t="inlineStr">
-        <is>
-          <t>高山岳</t>
-        </is>
-      </c>
-      <c r="L3" s="10" t="inlineStr">
-        <is>
-          <t>宮路愛</t>
-        </is>
-      </c>
       <c r="M3" s="10" t="inlineStr">
         <is>
+          <t>金上平</t>
+        </is>
+      </c>
+      <c r="N3" s="10" t="inlineStr">
+        <is>
           <t>藤田法成</t>
-        </is>
-      </c>
-      <c r="N3" s="10" t="inlineStr">
-        <is>
-          <t>金上平</t>
         </is>
       </c>
     </row>
@@ -1624,57 +1624,57 @@
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
+          <t>板倉芽生</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
           <t>山田恵美</t>
         </is>
       </c>
-      <c r="E3" s="10" t="inlineStr">
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>高山岳</t>
+        </is>
+      </c>
+      <c r="G3" s="10" t="inlineStr">
+        <is>
+          <t>宮路愛</t>
+        </is>
+      </c>
+      <c r="H3" s="10" t="inlineStr">
+        <is>
+          <t>若尾まい</t>
+        </is>
+      </c>
+      <c r="I3" s="10" t="inlineStr">
         <is>
           <t>永田千尋</t>
         </is>
       </c>
-      <c r="F3" s="10" t="inlineStr">
+      <c r="J3" s="10" t="inlineStr">
         <is>
           <t>鷹野かおり</t>
         </is>
       </c>
-      <c r="G3" s="10" t="inlineStr">
-        <is>
-          <t>若尾まい</t>
-        </is>
-      </c>
-      <c r="H3" s="10" t="inlineStr">
+      <c r="K3" s="10" t="inlineStr">
         <is>
           <t>大野リカ子</t>
         </is>
       </c>
-      <c r="I3" s="10" t="inlineStr">
+      <c r="L3" s="10" t="inlineStr">
         <is>
           <t>織田陽子</t>
         </is>
       </c>
-      <c r="J3" s="10" t="inlineStr">
-        <is>
-          <t>板倉芽生</t>
-        </is>
-      </c>
-      <c r="K3" s="10" t="inlineStr">
-        <is>
-          <t>高山岳</t>
-        </is>
-      </c>
-      <c r="L3" s="10" t="inlineStr">
-        <is>
-          <t>宮路愛</t>
-        </is>
-      </c>
       <c r="M3" s="10" t="inlineStr">
         <is>
+          <t>金上平</t>
+        </is>
+      </c>
+      <c r="N3" s="10" t="inlineStr">
+        <is>
           <t>藤田法成</t>
-        </is>
-      </c>
-      <c r="N3" s="10" t="inlineStr">
-        <is>
-          <t>金上平</t>
         </is>
       </c>
     </row>
@@ -2493,57 +2493,57 @@
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
+          <t>板倉芽生</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
           <t>山田恵美</t>
         </is>
       </c>
-      <c r="E3" s="10" t="inlineStr">
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>高山岳</t>
+        </is>
+      </c>
+      <c r="G3" s="10" t="inlineStr">
+        <is>
+          <t>宮路愛</t>
+        </is>
+      </c>
+      <c r="H3" s="10" t="inlineStr">
+        <is>
+          <t>若尾まい</t>
+        </is>
+      </c>
+      <c r="I3" s="10" t="inlineStr">
         <is>
           <t>永田千尋</t>
         </is>
       </c>
-      <c r="F3" s="10" t="inlineStr">
+      <c r="J3" s="10" t="inlineStr">
         <is>
           <t>鷹野かおり</t>
         </is>
       </c>
-      <c r="G3" s="10" t="inlineStr">
-        <is>
-          <t>若尾まい</t>
-        </is>
-      </c>
-      <c r="H3" s="10" t="inlineStr">
+      <c r="K3" s="10" t="inlineStr">
         <is>
           <t>大野リカ子</t>
         </is>
       </c>
-      <c r="I3" s="10" t="inlineStr">
+      <c r="L3" s="10" t="inlineStr">
         <is>
           <t>織田陽子</t>
         </is>
       </c>
-      <c r="J3" s="10" t="inlineStr">
-        <is>
-          <t>板倉芽生</t>
-        </is>
-      </c>
-      <c r="K3" s="10" t="inlineStr">
-        <is>
-          <t>高山岳</t>
-        </is>
-      </c>
-      <c r="L3" s="10" t="inlineStr">
-        <is>
-          <t>宮路愛</t>
-        </is>
-      </c>
       <c r="M3" s="10" t="inlineStr">
         <is>
+          <t>金上平</t>
+        </is>
+      </c>
+      <c r="N3" s="10" t="inlineStr">
+        <is>
           <t>藤田法成</t>
-        </is>
-      </c>
-      <c r="N3" s="10" t="inlineStr">
-        <is>
-          <t>金上平</t>
         </is>
       </c>
     </row>
@@ -3338,57 +3338,57 @@
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
+          <t>板倉芽生</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
           <t>山田恵美</t>
         </is>
       </c>
-      <c r="E3" s="10" t="inlineStr">
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>高山岳</t>
+        </is>
+      </c>
+      <c r="G3" s="10" t="inlineStr">
+        <is>
+          <t>宮路愛</t>
+        </is>
+      </c>
+      <c r="H3" s="10" t="inlineStr">
+        <is>
+          <t>若尾まい</t>
+        </is>
+      </c>
+      <c r="I3" s="10" t="inlineStr">
         <is>
           <t>永田千尋</t>
         </is>
       </c>
-      <c r="F3" s="10" t="inlineStr">
+      <c r="J3" s="10" t="inlineStr">
         <is>
           <t>鷹野かおり</t>
         </is>
       </c>
-      <c r="G3" s="10" t="inlineStr">
-        <is>
-          <t>若尾まい</t>
-        </is>
-      </c>
-      <c r="H3" s="10" t="inlineStr">
+      <c r="K3" s="10" t="inlineStr">
         <is>
           <t>大野リカ子</t>
         </is>
       </c>
-      <c r="I3" s="10" t="inlineStr">
+      <c r="L3" s="10" t="inlineStr">
         <is>
           <t>織田陽子</t>
         </is>
       </c>
-      <c r="J3" s="10" t="inlineStr">
-        <is>
-          <t>板倉芽生</t>
-        </is>
-      </c>
-      <c r="K3" s="10" t="inlineStr">
-        <is>
-          <t>高山岳</t>
-        </is>
-      </c>
-      <c r="L3" s="10" t="inlineStr">
-        <is>
-          <t>宮路愛</t>
-        </is>
-      </c>
       <c r="M3" s="10" t="inlineStr">
         <is>
+          <t>金上平</t>
+        </is>
+      </c>
+      <c r="N3" s="10" t="inlineStr">
+        <is>
           <t>藤田法成</t>
-        </is>
-      </c>
-      <c r="N3" s="10" t="inlineStr">
-        <is>
-          <t>金上平</t>
         </is>
       </c>
     </row>
@@ -4207,57 +4207,57 @@
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
+          <t>板倉芽生</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
           <t>山田恵美</t>
         </is>
       </c>
-      <c r="E3" s="10" t="inlineStr">
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>高山岳</t>
+        </is>
+      </c>
+      <c r="G3" s="10" t="inlineStr">
+        <is>
+          <t>宮路愛</t>
+        </is>
+      </c>
+      <c r="H3" s="10" t="inlineStr">
+        <is>
+          <t>若尾まい</t>
+        </is>
+      </c>
+      <c r="I3" s="10" t="inlineStr">
         <is>
           <t>永田千尋</t>
         </is>
       </c>
-      <c r="F3" s="10" t="inlineStr">
+      <c r="J3" s="10" t="inlineStr">
         <is>
           <t>鷹野かおり</t>
         </is>
       </c>
-      <c r="G3" s="10" t="inlineStr">
-        <is>
-          <t>若尾まい</t>
-        </is>
-      </c>
-      <c r="H3" s="10" t="inlineStr">
+      <c r="K3" s="10" t="inlineStr">
         <is>
           <t>大野リカ子</t>
         </is>
       </c>
-      <c r="I3" s="10" t="inlineStr">
+      <c r="L3" s="10" t="inlineStr">
         <is>
           <t>織田陽子</t>
         </is>
       </c>
-      <c r="J3" s="10" t="inlineStr">
-        <is>
-          <t>板倉芽生</t>
-        </is>
-      </c>
-      <c r="K3" s="10" t="inlineStr">
-        <is>
-          <t>高山岳</t>
-        </is>
-      </c>
-      <c r="L3" s="10" t="inlineStr">
-        <is>
-          <t>宮路愛</t>
-        </is>
-      </c>
       <c r="M3" s="10" t="inlineStr">
         <is>
+          <t>金上平</t>
+        </is>
+      </c>
+      <c r="N3" s="10" t="inlineStr">
+        <is>
           <t>藤田法成</t>
-        </is>
-      </c>
-      <c r="N3" s="10" t="inlineStr">
-        <is>
-          <t>金上平</t>
         </is>
       </c>
     </row>
@@ -5076,57 +5076,57 @@
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
+          <t>板倉芽生</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
           <t>山田恵美</t>
         </is>
       </c>
-      <c r="E3" s="10" t="inlineStr">
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>高山岳</t>
+        </is>
+      </c>
+      <c r="G3" s="10" t="inlineStr">
+        <is>
+          <t>宮路愛</t>
+        </is>
+      </c>
+      <c r="H3" s="10" t="inlineStr">
+        <is>
+          <t>若尾まい</t>
+        </is>
+      </c>
+      <c r="I3" s="10" t="inlineStr">
         <is>
           <t>永田千尋</t>
         </is>
       </c>
-      <c r="F3" s="10" t="inlineStr">
+      <c r="J3" s="10" t="inlineStr">
         <is>
           <t>鷹野かおり</t>
         </is>
       </c>
-      <c r="G3" s="10" t="inlineStr">
-        <is>
-          <t>若尾まい</t>
-        </is>
-      </c>
-      <c r="H3" s="10" t="inlineStr">
+      <c r="K3" s="10" t="inlineStr">
         <is>
           <t>大野リカ子</t>
         </is>
       </c>
-      <c r="I3" s="10" t="inlineStr">
+      <c r="L3" s="10" t="inlineStr">
         <is>
           <t>織田陽子</t>
         </is>
       </c>
-      <c r="J3" s="10" t="inlineStr">
-        <is>
-          <t>板倉芽生</t>
-        </is>
-      </c>
-      <c r="K3" s="10" t="inlineStr">
-        <is>
-          <t>高山岳</t>
-        </is>
-      </c>
-      <c r="L3" s="10" t="inlineStr">
-        <is>
-          <t>宮路愛</t>
-        </is>
-      </c>
       <c r="M3" s="10" t="inlineStr">
         <is>
+          <t>金上平</t>
+        </is>
+      </c>
+      <c r="N3" s="10" t="inlineStr">
+        <is>
           <t>藤田法成</t>
-        </is>
-      </c>
-      <c r="N3" s="10" t="inlineStr">
-        <is>
-          <t>金上平</t>
         </is>
       </c>
     </row>
@@ -5873,57 +5873,57 @@
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
+          <t>板倉芽生</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
           <t>山田恵美</t>
         </is>
       </c>
-      <c r="E3" s="10" t="inlineStr">
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>高山岳</t>
+        </is>
+      </c>
+      <c r="G3" s="10" t="inlineStr">
+        <is>
+          <t>宮路愛</t>
+        </is>
+      </c>
+      <c r="H3" s="10" t="inlineStr">
+        <is>
+          <t>若尾まい</t>
+        </is>
+      </c>
+      <c r="I3" s="10" t="inlineStr">
         <is>
           <t>永田千尋</t>
         </is>
       </c>
-      <c r="F3" s="10" t="inlineStr">
+      <c r="J3" s="10" t="inlineStr">
         <is>
           <t>鷹野かおり</t>
         </is>
       </c>
-      <c r="G3" s="10" t="inlineStr">
-        <is>
-          <t>若尾まい</t>
-        </is>
-      </c>
-      <c r="H3" s="10" t="inlineStr">
+      <c r="K3" s="10" t="inlineStr">
         <is>
           <t>大野リカ子</t>
         </is>
       </c>
-      <c r="I3" s="10" t="inlineStr">
+      <c r="L3" s="10" t="inlineStr">
         <is>
           <t>織田陽子</t>
         </is>
       </c>
-      <c r="J3" s="10" t="inlineStr">
-        <is>
-          <t>板倉芽生</t>
-        </is>
-      </c>
-      <c r="K3" s="10" t="inlineStr">
-        <is>
-          <t>高山岳</t>
-        </is>
-      </c>
-      <c r="L3" s="10" t="inlineStr">
-        <is>
-          <t>宮路愛</t>
-        </is>
-      </c>
       <c r="M3" s="10" t="inlineStr">
         <is>
+          <t>金上平</t>
+        </is>
+      </c>
+      <c r="N3" s="10" t="inlineStr">
+        <is>
           <t>藤田法成</t>
-        </is>
-      </c>
-      <c r="N3" s="10" t="inlineStr">
-        <is>
-          <t>金上平</t>
         </is>
       </c>
     </row>
@@ -6742,57 +6742,57 @@
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
+          <t>板倉芽生</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
           <t>山田恵美</t>
         </is>
       </c>
-      <c r="E3" s="10" t="inlineStr">
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>高山岳</t>
+        </is>
+      </c>
+      <c r="G3" s="10" t="inlineStr">
+        <is>
+          <t>宮路愛</t>
+        </is>
+      </c>
+      <c r="H3" s="10" t="inlineStr">
+        <is>
+          <t>若尾まい</t>
+        </is>
+      </c>
+      <c r="I3" s="10" t="inlineStr">
         <is>
           <t>永田千尋</t>
         </is>
       </c>
-      <c r="F3" s="10" t="inlineStr">
+      <c r="J3" s="10" t="inlineStr">
         <is>
           <t>鷹野かおり</t>
         </is>
       </c>
-      <c r="G3" s="10" t="inlineStr">
-        <is>
-          <t>若尾まい</t>
-        </is>
-      </c>
-      <c r="H3" s="10" t="inlineStr">
+      <c r="K3" s="10" t="inlineStr">
         <is>
           <t>大野リカ子</t>
         </is>
       </c>
-      <c r="I3" s="10" t="inlineStr">
+      <c r="L3" s="10" t="inlineStr">
         <is>
           <t>織田陽子</t>
         </is>
       </c>
-      <c r="J3" s="10" t="inlineStr">
-        <is>
-          <t>板倉芽生</t>
-        </is>
-      </c>
-      <c r="K3" s="10" t="inlineStr">
-        <is>
-          <t>高山岳</t>
-        </is>
-      </c>
-      <c r="L3" s="10" t="inlineStr">
-        <is>
-          <t>宮路愛</t>
-        </is>
-      </c>
       <c r="M3" s="10" t="inlineStr">
         <is>
+          <t>金上平</t>
+        </is>
+      </c>
+      <c r="N3" s="10" t="inlineStr">
+        <is>
           <t>藤田法成</t>
-        </is>
-      </c>
-      <c r="N3" s="10" t="inlineStr">
-        <is>
-          <t>金上平</t>
         </is>
       </c>
     </row>
@@ -7587,57 +7587,57 @@
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
+          <t>板倉芽生</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
           <t>山田恵美</t>
         </is>
       </c>
-      <c r="E3" s="10" t="inlineStr">
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>高山岳</t>
+        </is>
+      </c>
+      <c r="G3" s="10" t="inlineStr">
+        <is>
+          <t>宮路愛</t>
+        </is>
+      </c>
+      <c r="H3" s="10" t="inlineStr">
+        <is>
+          <t>若尾まい</t>
+        </is>
+      </c>
+      <c r="I3" s="10" t="inlineStr">
         <is>
           <t>永田千尋</t>
         </is>
       </c>
-      <c r="F3" s="10" t="inlineStr">
+      <c r="J3" s="10" t="inlineStr">
         <is>
           <t>鷹野かおり</t>
         </is>
       </c>
-      <c r="G3" s="10" t="inlineStr">
-        <is>
-          <t>若尾まい</t>
-        </is>
-      </c>
-      <c r="H3" s="10" t="inlineStr">
+      <c r="K3" s="10" t="inlineStr">
         <is>
           <t>大野リカ子</t>
         </is>
       </c>
-      <c r="I3" s="10" t="inlineStr">
+      <c r="L3" s="10" t="inlineStr">
         <is>
           <t>織田陽子</t>
         </is>
       </c>
-      <c r="J3" s="10" t="inlineStr">
-        <is>
-          <t>板倉芽生</t>
-        </is>
-      </c>
-      <c r="K3" s="10" t="inlineStr">
-        <is>
-          <t>高山岳</t>
-        </is>
-      </c>
-      <c r="L3" s="10" t="inlineStr">
-        <is>
-          <t>宮路愛</t>
-        </is>
-      </c>
       <c r="M3" s="10" t="inlineStr">
         <is>
+          <t>金上平</t>
+        </is>
+      </c>
+      <c r="N3" s="10" t="inlineStr">
+        <is>
           <t>藤田法成</t>
-        </is>
-      </c>
-      <c r="N3" s="10" t="inlineStr">
-        <is>
-          <t>金上平</t>
         </is>
       </c>
     </row>
@@ -8456,57 +8456,57 @@
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
+          <t>板倉芽生</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
           <t>山田恵美</t>
         </is>
       </c>
-      <c r="E3" s="10" t="inlineStr">
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>高山岳</t>
+        </is>
+      </c>
+      <c r="G3" s="10" t="inlineStr">
+        <is>
+          <t>宮路愛</t>
+        </is>
+      </c>
+      <c r="H3" s="10" t="inlineStr">
+        <is>
+          <t>若尾まい</t>
+        </is>
+      </c>
+      <c r="I3" s="10" t="inlineStr">
         <is>
           <t>永田千尋</t>
         </is>
       </c>
-      <c r="F3" s="10" t="inlineStr">
+      <c r="J3" s="10" t="inlineStr">
         <is>
           <t>鷹野かおり</t>
         </is>
       </c>
-      <c r="G3" s="10" t="inlineStr">
-        <is>
-          <t>若尾まい</t>
-        </is>
-      </c>
-      <c r="H3" s="10" t="inlineStr">
+      <c r="K3" s="10" t="inlineStr">
         <is>
           <t>大野リカ子</t>
         </is>
       </c>
-      <c r="I3" s="10" t="inlineStr">
+      <c r="L3" s="10" t="inlineStr">
         <is>
           <t>織田陽子</t>
         </is>
       </c>
-      <c r="J3" s="10" t="inlineStr">
-        <is>
-          <t>板倉芽生</t>
-        </is>
-      </c>
-      <c r="K3" s="10" t="inlineStr">
-        <is>
-          <t>高山岳</t>
-        </is>
-      </c>
-      <c r="L3" s="10" t="inlineStr">
-        <is>
-          <t>宮路愛</t>
-        </is>
-      </c>
       <c r="M3" s="10" t="inlineStr">
         <is>
+          <t>金上平</t>
+        </is>
+      </c>
+      <c r="N3" s="10" t="inlineStr">
+        <is>
           <t>藤田法成</t>
-        </is>
-      </c>
-      <c r="N3" s="10" t="inlineStr">
-        <is>
-          <t>金上平</t>
         </is>
       </c>
     </row>
@@ -9301,57 +9301,57 @@
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
+          <t>板倉芽生</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
           <t>山田恵美</t>
         </is>
       </c>
-      <c r="E3" s="10" t="inlineStr">
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>高山岳</t>
+        </is>
+      </c>
+      <c r="G3" s="10" t="inlineStr">
+        <is>
+          <t>宮路愛</t>
+        </is>
+      </c>
+      <c r="H3" s="10" t="inlineStr">
+        <is>
+          <t>若尾まい</t>
+        </is>
+      </c>
+      <c r="I3" s="10" t="inlineStr">
         <is>
           <t>永田千尋</t>
         </is>
       </c>
-      <c r="F3" s="10" t="inlineStr">
+      <c r="J3" s="10" t="inlineStr">
         <is>
           <t>鷹野かおり</t>
         </is>
       </c>
-      <c r="G3" s="10" t="inlineStr">
-        <is>
-          <t>若尾まい</t>
-        </is>
-      </c>
-      <c r="H3" s="10" t="inlineStr">
+      <c r="K3" s="10" t="inlineStr">
         <is>
           <t>大野リカ子</t>
         </is>
       </c>
-      <c r="I3" s="10" t="inlineStr">
+      <c r="L3" s="10" t="inlineStr">
         <is>
           <t>織田陽子</t>
         </is>
       </c>
-      <c r="J3" s="10" t="inlineStr">
-        <is>
-          <t>板倉芽生</t>
-        </is>
-      </c>
-      <c r="K3" s="10" t="inlineStr">
-        <is>
-          <t>高山岳</t>
-        </is>
-      </c>
-      <c r="L3" s="10" t="inlineStr">
-        <is>
-          <t>宮路愛</t>
-        </is>
-      </c>
       <c r="M3" s="10" t="inlineStr">
         <is>
+          <t>金上平</t>
+        </is>
+      </c>
+      <c r="N3" s="10" t="inlineStr">
+        <is>
           <t>藤田法成</t>
-        </is>
-      </c>
-      <c r="N3" s="10" t="inlineStr">
-        <is>
-          <t>金上平</t>
         </is>
       </c>
     </row>
@@ -10170,57 +10170,57 @@
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
+          <t>板倉芽生</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
           <t>山田恵美</t>
         </is>
       </c>
-      <c r="E3" s="10" t="inlineStr">
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>高山岳</t>
+        </is>
+      </c>
+      <c r="G3" s="10" t="inlineStr">
+        <is>
+          <t>宮路愛</t>
+        </is>
+      </c>
+      <c r="H3" s="10" t="inlineStr">
+        <is>
+          <t>若尾まい</t>
+        </is>
+      </c>
+      <c r="I3" s="10" t="inlineStr">
         <is>
           <t>永田千尋</t>
         </is>
       </c>
-      <c r="F3" s="10" t="inlineStr">
+      <c r="J3" s="10" t="inlineStr">
         <is>
           <t>鷹野かおり</t>
         </is>
       </c>
-      <c r="G3" s="10" t="inlineStr">
-        <is>
-          <t>若尾まい</t>
-        </is>
-      </c>
-      <c r="H3" s="10" t="inlineStr">
+      <c r="K3" s="10" t="inlineStr">
         <is>
           <t>大野リカ子</t>
         </is>
       </c>
-      <c r="I3" s="10" t="inlineStr">
+      <c r="L3" s="10" t="inlineStr">
         <is>
           <t>織田陽子</t>
         </is>
       </c>
-      <c r="J3" s="10" t="inlineStr">
-        <is>
-          <t>板倉芽生</t>
-        </is>
-      </c>
-      <c r="K3" s="10" t="inlineStr">
-        <is>
-          <t>高山岳</t>
-        </is>
-      </c>
-      <c r="L3" s="10" t="inlineStr">
-        <is>
-          <t>宮路愛</t>
-        </is>
-      </c>
       <c r="M3" s="10" t="inlineStr">
         <is>
+          <t>金上平</t>
+        </is>
+      </c>
+      <c r="N3" s="10" t="inlineStr">
+        <is>
           <t>藤田法成</t>
-        </is>
-      </c>
-      <c r="N3" s="10" t="inlineStr">
-        <is>
-          <t>金上平</t>
         </is>
       </c>
     </row>

</xml_diff>